<commit_message>
Enrich resume assets with OPC statistics
</commit_message>
<xml_diff>
--- a/resume-assets/achievement-library-public.xlsx
+++ b/resume-assets/achievement-library-public.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="Re6ff500c04664ed9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成就素材库" sheetId="2" r:id="Rb1dc4fedf27d453b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="标签词典" sheetId="3" r:id="R8df20a515a0446cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R7f0c732c02494006"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成就素材库" sheetId="2" r:id="R17e2a512545b49bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="标签词典" sheetId="3" r:id="R72990b1f0b6b4b53"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -272,7 +272,7 @@
         <x:v>素材总数</x:v>
       </x:c>
       <x:c r="B4" t="n">
-        <x:v>25</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -280,7 +280,7 @@
         <x:v>A 级素材</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:v>14</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -288,7 +288,7 @@
         <x:v>OPC 相关素材</x:v>
       </x:c>
       <x:c r="B6" t="n">
-        <x:v>1</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -411,7 +411,9 @@
       <x:c r="J2" t="str">
         <x:v>减少人工翻找、重复确认和会议对齐时间。</x:v>
       </x:c>
-      <x:c r="K2" t="str"/>
+      <x:c r="K2" t="str">
+        <x:v>20 个项目/产物组；104 个候选线索；14 个业务域；116 条 session 原文证据；113 个独立 session；2000 条文件证据采样；129 个 output 产物；6 个 H5 Demo</x:v>
+      </x:c>
       <x:c r="L2" t="str">
         <x:v>业务架构, 证据化诊断, 复杂需求拆解, 项目对齐</x:v>
       </x:c>
@@ -463,7 +465,7 @@
         <x:v>形成 Figma Make 工作区规则和供应商管理规则。</x:v>
       </x:c>
       <x:c r="K3" t="str">
-        <x:v>6 个 OPC 工作区</x:v>
+        <x:v>8 份规则文档；101 条带产物路径的 session 证据；952 次路径/产物命中；6 个公开 H5 Demo</x:v>
       </x:c>
       <x:c r="L3" t="str">
         <x:v>Figma 治理, 验收规则, 状态模型, 交互诊断</x:v>
@@ -1695,6 +1697,271 @@
       </x:c>
       <x:c r="Q26" t="str">
         <x:v>待补充</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>A026</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>AI 产品/项目</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>OPC 项目证据盘点与经历证明库</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>2026.03-2026.06</x:v>
+      </x:c>
+      <x:c r="F27" t="str">
+        <x:v>AI Native 产品经理 / 项目统筹</x:v>
+      </x:c>
+      <x:c r="G27" t="str">
+        <x:v>把分散在会议、Figma Make、XMind、Excel、H5、前端包和 Codex session 里的 OPC 项目材料整理成可证明经历的素材库、案例库和证据索引。</x:v>
+      </x:c>
+      <x:c r="H27" t="str">
+        <x:v>OPC 不是单一代码仓库，证据分散在本机、macmini、Figma 包、证据库和 session 里；不统计就很难写成有说服力的简历经历。</x:v>
+      </x:c>
+      <x:c r="I27" t="str">
+        <x:v>先做项目候选清单，再从 session 原文抽请求、结论和产物路径，最后按业务产品、前端包、自动化、可视化、沟通研究、GitHub 六层重组。</x:v>
+      </x:c>
+      <x:c r="J27" t="str">
+        <x:v>形成可直接进入简历和 GitHub 作品集的项目地图、功能模块清单、统计证据页和公开案例库。</x:v>
+      </x:c>
+      <x:c r="K27" t="str">
+        <x:v>20 个项目/产物组；104 个候选线索；14 个业务域；116 条 session 原文证据；113 个独立 session；2000 条文件证据采样；129 个 output 产物；6 个 H5 Demo</x:v>
+      </x:c>
+      <x:c r="L27" t="str">
+        <x:v>复杂项目盘点, 证据化项目管理, AI 工作流, 项目经历证明, GitHub 作品集</x:v>
+      </x:c>
+      <x:c r="M27" t="str">
+        <x:v>AI Native 产品经理, 项目经理, 解决方案产品, 业务分析, AI 应用架构师</x:v>
+      </x:c>
+      <x:c r="N27" t="str">
+        <x:v>围绕 OPC 项目经历，统计并整理 20 个项目/产物组、104 个候选线索、116 条 session 原文证据和 2000 条文件证据采样，沉淀为项目地图、功能模块清单、证据索引和公开 GitHub 案例库。</x:v>
+      </x:c>
+      <x:c r="O27" t="str">
+        <x:v>Audited and structured OPC project evidence into 20 project groups, 104 candidate leads, 116 session-evidence rows and 2000 file-evidence samples, turning fragmented work into a GitHub casebook and resume asset library.</x:v>
+      </x:c>
+      <x:c r="P27" t="str">
+        <x:v>已统计</x:v>
+      </x:c>
+      <x:c r="Q27" t="str">
+        <x:v>可用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>A027</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>产品架构/需求拆解</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>OPC 业务功能模块拆解</x:v>
+      </x:c>
+      <x:c r="E28" t="str">
+        <x:v>2026.03-2026.06</x:v>
+      </x:c>
+      <x:c r="F28" t="str">
+        <x:v>AI Native 产品经理 / 业务架构整理</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>把业务线索拆成可筛选、可复用、可对齐的功能模块清单，并标注证据强度和核心证据来源。</x:v>
+      </x:c>
+      <x:c r="H28" t="str">
+        <x:v>OPC 涉及多角色、多链路、多工作区，单靠项目名看不出能力；必须拆到功能颗粒，才能证明复杂需求理解和产品架构能力。</x:v>
+      </x:c>
+      <x:c r="I28" t="str">
+        <x:v>按业务域归档模块，再把模块关联到项目地图、候选表、session 原文证据和 output 产物。</x:v>
+      </x:c>
+      <x:c r="J28" t="str">
+        <x:v>沉淀 428 行功能模块清单，为简历 bullet、面试讲述和作品集页面提供可追溯素材。</x:v>
+      </x:c>
+      <x:c r="K28" t="str">
+        <x:v>14 个业务域；428 行功能模块清单；20 个项目/产物组；6 层项目地图</x:v>
+      </x:c>
+      <x:c r="L28" t="str">
+        <x:v>产品架构, 复杂需求拆解, 业务模块化, 证据归档, 功能清单</x:v>
+      </x:c>
+      <x:c r="M28" t="str">
+        <x:v>产品经理, 业务分析, 解决方案产品, 项目交付</x:v>
+      </x:c>
+      <x:c r="N28" t="str">
+        <x:v>将 OPC 复杂业务拆成 14 个业务域和 20 个项目/产物组，覆盖平台配置、招商授权、供应商、分润、营销推广和 CPS 履约等模块，并沉淀 428 行功能模块清单。</x:v>
+      </x:c>
+      <x:c r="O28" t="str">
+        <x:v>Broke down OPC complex business architecture into 14 business domains and 20 project/output groups, producing a 428-line module inventory across listing configuration, channel permissions, supplier, profit-sharing, marketing and fulfillment flows.</x:v>
+      </x:c>
+      <x:c r="P28" t="str">
+        <x:v>已统计</x:v>
+      </x:c>
+      <x:c r="Q28" t="str">
+        <x:v>可用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>A028</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>产品文档/开发指令</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>OPC 系统需求总包与开发指令</x:v>
+      </x:c>
+      <x:c r="E29" t="str">
+        <x:v>2026.06</x:v>
+      </x:c>
+      <x:c r="F29" t="str">
+        <x:v>产品经理 / 需求包整理</x:v>
+      </x:c>
+      <x:c r="G29" t="str">
+        <x:v>把 OPC 总体业务从散落材料整理为总览、模块表、流程、页面规划、角色权限、功能需求、开发指令和喂数规则。</x:v>
+      </x:c>
+      <x:c r="H29" t="str">
+        <x:v>复杂系统如果没有统一需求包，开发、设计和业务判断会反复切换口径。</x:v>
+      </x:c>
+      <x:c r="I29" t="str">
+        <x:v>用总规划页、功能索引、多包功能归属和开发指令把业务材料压成可执行包。</x:v>
+      </x:c>
+      <x:c r="J29" t="str">
+        <x:v>形成能直接给团队阅读和执行的 OPC 系统需求总包。</x:v>
+      </x:c>
+      <x:c r="K29" t="str">
+        <x:v>11 个需求总包文件；包含项目总览、业务模块总表、核心业务流程、页面规划、角色权限、功能需求、Codex开发指令、FigmaMake喂数规则</x:v>
+      </x:c>
+      <x:c r="L29" t="str">
+        <x:v>PRD, 页面规划, 开发指令, Figma Make 喂数, 需求包设计</x:v>
+      </x:c>
+      <x:c r="M29" t="str">
+        <x:v>AI Native 产品经理, 产品经理, 项目交付, 解决方案产品</x:v>
+      </x:c>
+      <x:c r="N29" t="str">
+        <x:v>整理 OPC 系统需求总包，将项目总览、业务模块、核心流程、页面规划、角色权限、功能需求、Codex 开发指令和 Figma Make 喂数规则沉淀为 11 个可执行文件。</x:v>
+      </x:c>
+      <x:c r="O29" t="str">
+        <x:v>Packaged OPC requirements into 11 executable planning files, covering overview, modules, workflows, page plans, permissions, feature requirements, Codex instructions and Figma Make input rules.</x:v>
+      </x:c>
+      <x:c r="P29" t="str">
+        <x:v>已统计</x:v>
+      </x:c>
+      <x:c r="Q29" t="str">
+        <x:v>可用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>A029</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>Figma Make 治理</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>OPC Figma Make 工作区规则与证据自动化</x:v>
+      </x:c>
+      <x:c r="E30" t="str">
+        <x:v>2026.05-2026.06</x:v>
+      </x:c>
+      <x:c r="F30" t="str">
+        <x:v>AI Native 产品经理 / Figma Make 协同</x:v>
+      </x:c>
+      <x:c r="G30" t="str">
+        <x:v>把工作区规则、包级变更、页面差异、PM 判断、版本归档和每日增量证据串成可追踪流程。</x:v>
+      </x:c>
+      <x:c r="H30" t="str">
+        <x:v>Figma Make 生成和修改频繁，如果没有包、页面、版本、PM 判断和证据链，容易误判完成度。</x:v>
+      </x:c>
+      <x:c r="I30" t="str">
+        <x:v>通过规则文档、包级变更总控、每日抓取、02/04 同步口径和版本归档建立治理方式。</x:v>
+      </x:c>
+      <x:c r="J30" t="str">
+        <x:v>形成 Figma Make 工作区规则、包级变更判断口径和自动化证据链。</x:v>
+      </x:c>
+      <x:c r="K30" t="str">
+        <x:v>8 份规则文档；101 条带产物路径的 session 证据；952 次路径/产物命中；6 个公开 H5 Demo</x:v>
+      </x:c>
+      <x:c r="L30" t="str">
+        <x:v>Figma Make 治理, 版本归档, 自动化证据链, PM 判断, 交付状态模型</x:v>
+      </x:c>
+      <x:c r="M30" t="str">
+        <x:v>Figma Make 产品/运营, AI Native 产品经理, 交付 PM, 产品经理</x:v>
+      </x:c>
+      <x:c r="N30" t="str">
+        <x:v>为 OPC Figma Make 多工作区建立规则和证据链，沉淀 8 份工作区规则文档，从 session 原文中抽取 101 条带产物路径的证据记录和 952 次路径/产物命中，用于判断包级变更、PM 确认和版本归档。</x:v>
+      </x:c>
+      <x:c r="O30" t="str">
+        <x:v>Established Figma Make governance for OPC workspaces with 8 rule documents and extracted 101 artifact-backed session records with 952 path/artifact hits to support package-level change tracking and PM review.</x:v>
+      </x:c>
+      <x:c r="P30" t="str">
+        <x:v>已统计</x:v>
+      </x:c>
+      <x:c r="Q30" t="str">
+        <x:v>可用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>A030</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>作品集/公开表达</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>OPC GitHub 公开项目案例库</x:v>
+      </x:c>
+      <x:c r="E31" t="str">
+        <x:v>2026.06</x:v>
+      </x:c>
+      <x:c r="F31" t="str">
+        <x:v>AI Native 产品经理 / 作品集整理</x:v>
+      </x:c>
+      <x:c r="G31" t="str">
+        <x:v>把内部项目材料整理成公开可读的 casebook、H5 Demo、脱敏证据索引和成就素材库公开版。</x:v>
+      </x:c>
+      <x:c r="H31" t="str">
+        <x:v>项目经历需要能被外部快速理解，不能只堆本地原始材料；同时公开仓必须控制敏感信息和大文件。</x:v>
+      </x:c>
+      <x:c r="I31" t="str">
+        <x:v>从原始 3.7G 工作区里筛选可公开材料，删除音频、模型、日志、原始 API/Feishu JSON、聊天原文和本机路径。</x:v>
+      </x:c>
+      <x:c r="J31" t="str">
+        <x:v>形成可直接发给招聘方或合作方查看的公开项目案例库和 Pages 展示页。</x:v>
+      </x:c>
+      <x:c r="K31" t="str">
+        <x:v>23 个公开文件；6 个 H5 Demo；仓库 约 2.7 MB；0 个超过 25MB 文件；敏感路径/凭证扫描 0 命中</x:v>
+      </x:c>
+      <x:c r="L31" t="str">
+        <x:v>GitHub 作品集, 脱敏, 项目包装, 公开表达, 证据索引</x:v>
+      </x:c>
+      <x:c r="M31" t="str">
+        <x:v>AI Native 产品经理, 产品经理, 解决方案产品, 项目交付</x:v>
+      </x:c>
+      <x:c r="N31" t="str">
+        <x:v>把 OPC 原始工作区整理为公开 GitHub 项目案例库，筛选出 23 个公开文件和 6 个 H5 Demo，并完成大文件、路径和凭证扫描，形成可对外展示的项目经历证明。</x:v>
+      </x:c>
+      <x:c r="O31" t="str">
+        <x:v>Converted the OPC workspace into a public GitHub casebook with 23 files and 6 H5 demos, excluding raw logs, audio, API data and credentials while preserving portfolio-ready evidence.</x:v>
+      </x:c>
+      <x:c r="P31" t="str">
+        <x:v>已统计</x:v>
+      </x:c>
+      <x:c r="Q31" t="str">
+        <x:v>可用</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Expand engineering evidence archive
</commit_message>
<xml_diff>
--- a/resume-assets/achievement-library-public.xlsx
+++ b/resume-assets/achievement-library-public.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R7f0c732c02494006"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成就素材库" sheetId="2" r:id="R17e2a512545b49bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="标签词典" sheetId="3" r:id="R72990b1f0b6b4b53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R3102e4b9e7e145be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成就素材库" sheetId="2" r:id="Rb1f10f8fa17c40d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="标签词典" sheetId="3" r:id="Rde8a1d433fdf4058"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1943,7 +1943,7 @@
         <x:v>形成可直接发给招聘方或合作方查看的公开项目案例库和 Pages 展示页。</x:v>
       </x:c>
       <x:c r="K31" t="str">
-        <x:v>23 个公开文件；6 个 H5 Demo；仓库 约 2.7 MB；0 个超过 25MB 文件；敏感路径/凭证扫描 0 命中</x:v>
+        <x:v>38 个公开文件；6 个 H5 Demo；公开内容约 1.9 MB；0 个超过 25MB 文件；敏感路径/凭证扫描 0 命中；13 条失败复盘条目</x:v>
       </x:c>
       <x:c r="L31" t="str">
         <x:v>GitHub 作品集, 脱敏, 项目包装, 公开表达, 证据索引</x:v>
@@ -1952,10 +1952,10 @@
         <x:v>AI Native 产品经理, 产品经理, 解决方案产品, 项目交付</x:v>
       </x:c>
       <x:c r="N31" t="str">
-        <x:v>把 OPC 原始工作区整理为公开 GitHub 项目案例库，筛选出 23 个公开文件和 6 个 H5 Demo，并完成大文件、路径和凭证扫描，形成可对外展示的项目经历证明。</x:v>
+        <x:v>把 OPC 原始工作区整理为公开 GitHub 工程证据库，筛选出 38 个公开文件和 6 个 H5 Demo，补充 13 条失败复盘，并完成大文件、路径和凭证扫描，形成可对外展示的项目经历证明。</x:v>
       </x:c>
       <x:c r="O31" t="str">
-        <x:v>Converted the OPC workspace into a public GitHub casebook with 23 files and 6 H5 demos, excluding raw logs, audio, API data and credentials while preserving portfolio-ready evidence.</x:v>
+        <x:v>Converted the OPC workspace into a public GitHub engineering evidence archive with 38 public files, 6 H5 demos and 13 documented failure-review items, excluding raw logs, audio, API data and credentials while preserving portfolio-ready proof.</x:v>
       </x:c>
       <x:c r="P31" t="str">
         <x:v>已统计</x:v>

</xml_diff>

<commit_message>
Localize public archive docs to Chinese
</commit_message>
<xml_diff>
--- a/resume-assets/achievement-library-public.xlsx
+++ b/resume-assets/achievement-library-public.xlsx
@@ -10,10 +10,11 @@
     <sheet name="概览" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="成就素材库" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="标签词典" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="OPC利益测算" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'成就素材库'!$A$1:$H$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'标签词典'!$A$1:$B$146</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'成就素材库'!$A$1:$H$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'标签词典'!$A$1:$B$150</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -80,7 +81,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -462,7 +463,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>OPC Project Casebook</t>
+          <t>OPC 项目案例库</t>
         </is>
       </c>
     </row>
@@ -473,7 +474,7 @@
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3">
@@ -503,7 +504,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>新增收益口径</t>
+          <t>收益口径</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -535,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1964,8 +1965,50 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>A034</t>
+        </is>
+      </c>
+      <c r="B35" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C35" s="1" t="inlineStr">
+        <is>
+          <t>商业测算/方法论</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="inlineStr">
+        <is>
+          <t>OPC 商业影响测算方法论</t>
+        </is>
+      </c>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>AI Native 产品经理 / 业务分析</t>
+        </is>
+      </c>
+      <c r="F35" s="1" t="inlineStr">
+        <is>
+          <t>四层数据等级；反事实比较；5个公式；低/高区间；可写 62.1-144.8 小时、¥0.75万-¥3.42万；不可硬写真实GMV/客户</t>
+        </is>
+      </c>
+      <c r="G35" s="1" t="inlineStr">
+        <is>
+          <t>商业影响测算, 反事实比较, 成本节约, 证据分级, 简历表达</t>
+        </is>
+      </c>
+      <c r="H35" s="1" t="inlineStr">
+        <is>
+          <t>建立 OPC 商业影响测算方法论：先把事实数据分层，再用“没有证据库 vs 有证据库”的反事实比较计算过程收益，最后用公开人力成本折算为 ¥0.75万-¥3.42万 人工成本节约；对 GMV、客户增长保持公式边界，不做无证据声称。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H34"/>
+  <autoFilter ref="A1:H35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1976,7 +2019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B146"/>
+  <dimension ref="A1:B150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2008,17 +2051,17 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Figma Make 治理</t>
+          <t>成本节约</t>
         </is>
       </c>
       <c r="B3" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>GitHub 作品集</t>
+          <t>Figma Make 治理</t>
         </is>
       </c>
       <c r="B4" s="1" t="n">
@@ -2028,7 +2071,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>PRD</t>
+          <t>GitHub 作品集</t>
         </is>
       </c>
       <c r="B5" s="1" t="n">
@@ -2038,7 +2081,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>复杂需求拆解</t>
+          <t>PRD</t>
         </is>
       </c>
       <c r="B6" s="1" t="n">
@@ -2048,7 +2091,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>成本节约</t>
+          <t>复杂需求拆解</t>
         </is>
       </c>
       <c r="B7" s="1" t="n">
@@ -2618,7 +2661,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>可运维化</t>
+          <t>反事实比较</t>
         </is>
       </c>
       <c r="B64" s="1" t="n">
@@ -2628,7 +2671,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>咨询产品化</t>
+          <t>可运维化</t>
         </is>
       </c>
       <c r="B65" s="1" t="n">
@@ -2638,7 +2681,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>商业化包装</t>
+          <t>咨询产品化</t>
         </is>
       </c>
       <c r="B66" s="1" t="n">
@@ -2648,7 +2691,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>商业模式分析</t>
+          <t>商业化包装</t>
         </is>
       </c>
       <c r="B67" s="1" t="n">
@@ -2658,7 +2701,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>商业测算</t>
+          <t>商业影响测算</t>
         </is>
       </c>
       <c r="B68" s="1" t="n">
@@ -2668,7 +2711,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>商品上架</t>
+          <t>商业模式分析</t>
         </is>
       </c>
       <c r="B69" s="1" t="n">
@@ -2678,7 +2721,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>团队管理</t>
+          <t>商业测算</t>
         </is>
       </c>
       <c r="B70" s="1" t="n">
@@ -2688,7 +2731,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>增长产品</t>
+          <t>商品上架</t>
         </is>
       </c>
       <c r="B71" s="1" t="n">
@@ -2698,7 +2741,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>复杂项目盘点</t>
+          <t>团队管理</t>
         </is>
       </c>
       <c r="B72" s="1" t="n">
@@ -2708,7 +2751,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>复杂项目管理</t>
+          <t>增长产品</t>
         </is>
       </c>
       <c r="B73" s="1" t="n">
@@ -2718,7 +2761,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>外联节奏</t>
+          <t>复杂项目盘点</t>
         </is>
       </c>
       <c r="B74" s="1" t="n">
@@ -2728,7 +2771,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>大型活动控场</t>
+          <t>复杂项目管理</t>
         </is>
       </c>
       <c r="B75" s="1" t="n">
@@ -2738,7 +2781,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>大型活动统筹</t>
+          <t>外联节奏</t>
         </is>
       </c>
       <c r="B76" s="1" t="n">
@@ -2748,7 +2791,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>失败复盘</t>
+          <t>大型活动控场</t>
         </is>
       </c>
       <c r="B77" s="1" t="n">
@@ -2758,7 +2801,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>定价</t>
+          <t>大型活动统筹</t>
         </is>
       </c>
       <c r="B78" s="1" t="n">
@@ -2768,7 +2811,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>审批协调</t>
+          <t>失败复盘</t>
         </is>
       </c>
       <c r="B79" s="1" t="n">
@@ -2778,7 +2821,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>客户互动</t>
+          <t>定价</t>
         </is>
       </c>
       <c r="B80" s="1" t="n">
@@ -2788,7 +2831,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>宣传内容</t>
+          <t>审批协调</t>
         </is>
       </c>
       <c r="B81" s="1" t="n">
@@ -2798,7 +2841,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>并行任务</t>
+          <t>客户互动</t>
         </is>
       </c>
       <c r="B82" s="1" t="n">
@@ -2808,7 +2851,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>应急重排</t>
+          <t>宣传内容</t>
         </is>
       </c>
       <c r="B83" s="1" t="n">
@@ -2818,7 +2861,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>开发指令</t>
+          <t>并行任务</t>
         </is>
       </c>
       <c r="B84" s="1" t="n">
@@ -2828,7 +2871,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>异常诊断</t>
+          <t>应急重排</t>
         </is>
       </c>
       <c r="B85" s="1" t="n">
@@ -2838,7 +2881,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>成本节省</t>
+          <t>开发指令</t>
         </is>
       </c>
       <c r="B86" s="1" t="n">
@@ -2848,7 +2891,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>打包交付</t>
+          <t>异常诊断</t>
         </is>
       </c>
       <c r="B87" s="1" t="n">
@@ -2858,7 +2901,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>报告产品化</t>
+          <t>成本节省</t>
         </is>
       </c>
       <c r="B88" s="1" t="n">
@@ -2868,7 +2911,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>指标口径</t>
+          <t>打包交付</t>
         </is>
       </c>
       <c r="B89" s="1" t="n">
@@ -2878,7 +2921,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>排障 Playbook</t>
+          <t>报告产品化</t>
         </is>
       </c>
       <c r="B90" s="1" t="n">
@@ -2888,7 +2931,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>摘要</t>
+          <t>指标口径</t>
         </is>
       </c>
       <c r="B91" s="1" t="n">
@@ -2898,7 +2941,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>数据字段</t>
+          <t>排障 Playbook</t>
         </is>
       </c>
       <c r="B92" s="1" t="n">
@@ -2908,7 +2951,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>数据驱动运营</t>
+          <t>摘要</t>
         </is>
       </c>
       <c r="B93" s="1" t="n">
@@ -2918,7 +2961,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>文档自动化</t>
+          <t>数据字段</t>
         </is>
       </c>
       <c r="B94" s="1" t="n">
@@ -2928,7 +2971,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>方案沟通</t>
+          <t>数据驱动运营</t>
         </is>
       </c>
       <c r="B95" s="1" t="n">
@@ -2938,7 +2981,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>方案蓝图</t>
+          <t>文档自动化</t>
         </is>
       </c>
       <c r="B96" s="1" t="n">
@@ -2948,7 +2991,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>服务报告</t>
+          <t>方案沟通</t>
         </is>
       </c>
       <c r="B97" s="1" t="n">
@@ -2958,7 +3001,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>本地模型</t>
+          <t>方案蓝图</t>
         </is>
       </c>
       <c r="B98" s="1" t="n">
@@ -2968,7 +3011,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>权益设计</t>
+          <t>服务报告</t>
         </is>
       </c>
       <c r="B99" s="1" t="n">
@@ -2978,7 +3021,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>校园组织</t>
+          <t>本地模型</t>
         </is>
       </c>
       <c r="B100" s="1" t="n">
@@ -2988,7 +3031,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>校园营销</t>
+          <t>权益设计</t>
         </is>
       </c>
       <c r="B101" s="1" t="n">
@@ -2998,7 +3041,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>桌面产品</t>
+          <t>校园组织</t>
         </is>
       </c>
       <c r="B102" s="1" t="n">
@@ -3008,7 +3051,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>桌面工具设计</t>
+          <t>校园营销</t>
         </is>
       </c>
       <c r="B103" s="1" t="n">
@@ -3018,7 +3061,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>活动主理</t>
+          <t>桌面产品</t>
         </is>
       </c>
       <c r="B104" s="1" t="n">
@@ -3028,7 +3071,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>活动推广</t>
+          <t>桌面工具设计</t>
         </is>
       </c>
       <c r="B105" s="1" t="n">
@@ -3038,7 +3081,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>版本归档</t>
+          <t>活动主理</t>
         </is>
       </c>
       <c r="B106" s="1" t="n">
@@ -3048,7 +3091,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>状态模型</t>
+          <t>活动推广</t>
         </is>
       </c>
       <c r="B107" s="1" t="n">
@@ -3058,7 +3101,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>状态表</t>
+          <t>版本归档</t>
         </is>
       </c>
       <c r="B108" s="1" t="n">
@@ -3068,7 +3111,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>现场主持</t>
+          <t>状态模型</t>
         </is>
       </c>
       <c r="B109" s="1" t="n">
@@ -3078,7 +3121,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>现场执行</t>
+          <t>状态表</t>
         </is>
       </c>
       <c r="B110" s="1" t="n">
@@ -3088,7 +3131,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>现场控场</t>
+          <t>现场主持</t>
         </is>
       </c>
       <c r="B111" s="1" t="n">
@@ -3098,7 +3141,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>用户体验</t>
+          <t>现场执行</t>
         </is>
       </c>
       <c r="B112" s="1" t="n">
@@ -3108,7 +3151,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>用户支持</t>
+          <t>现场控场</t>
         </is>
       </c>
       <c r="B113" s="1" t="n">
@@ -3118,7 +3161,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>用户获取</t>
+          <t>用户体验</t>
         </is>
       </c>
       <c r="B114" s="1" t="n">
@@ -3128,7 +3171,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>私域运营</t>
+          <t>用户支持</t>
         </is>
       </c>
       <c r="B115" s="1" t="n">
@@ -3138,7 +3181,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>竞品分析</t>
+          <t>用户获取</t>
         </is>
       </c>
       <c r="B116" s="1" t="n">
@@ -3148,7 +3191,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>线下运营</t>
+          <t>私域运营</t>
         </is>
       </c>
       <c r="B117" s="1" t="n">
@@ -3158,7 +3201,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>结构化访谈</t>
+          <t>竞品分析</t>
         </is>
       </c>
       <c r="B118" s="1" t="n">
@@ -3168,7 +3211,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>脱敏</t>
+          <t>简历表达</t>
         </is>
       </c>
       <c r="B119" s="1" t="n">
@@ -3178,7 +3221,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>自动化信息流</t>
+          <t>线下运营</t>
         </is>
       </c>
       <c r="B120" s="1" t="n">
@@ -3188,7 +3231,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>自动化证据链</t>
+          <t>结构化访谈</t>
         </is>
       </c>
       <c r="B121" s="1" t="n">
@@ -3198,7 +3241,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>英语沟通</t>
+          <t>脱敏</t>
         </is>
       </c>
       <c r="B122" s="1" t="n">
@@ -3208,7 +3251,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>规则库</t>
+          <t>自动化信息流</t>
         </is>
       </c>
       <c r="B123" s="1" t="n">
@@ -3218,7 +3261,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>视频制作</t>
+          <t>自动化证据链</t>
         </is>
       </c>
       <c r="B124" s="1" t="n">
@@ -3228,7 +3271,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>证据化诊断</t>
+          <t>英语沟通</t>
         </is>
       </c>
       <c r="B125" s="1" t="n">
@@ -3238,7 +3281,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>证据化项目管理</t>
+          <t>规则库</t>
         </is>
       </c>
       <c r="B126" s="1" t="n">
@@ -3248,7 +3291,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>证据归档</t>
+          <t>视频制作</t>
         </is>
       </c>
       <c r="B127" s="1" t="n">
@@ -3258,7 +3301,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>证据索引</t>
+          <t>证据分级</t>
         </is>
       </c>
       <c r="B128" s="1" t="n">
@@ -3268,7 +3311,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>话题设计</t>
+          <t>证据化诊断</t>
         </is>
       </c>
       <c r="B129" s="1" t="n">
@@ -3278,7 +3321,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>资源整合</t>
+          <t>证据化项目管理</t>
         </is>
       </c>
       <c r="B130" s="1" t="n">
@@ -3288,7 +3331,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>赞助沟通</t>
+          <t>证据归档</t>
         </is>
       </c>
       <c r="B131" s="1" t="n">
@@ -3298,7 +3341,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>跨文化引导</t>
+          <t>证据索引</t>
         </is>
       </c>
       <c r="B132" s="1" t="n">
@@ -3308,7 +3351,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>转化路径</t>
+          <t>话题设计</t>
         </is>
       </c>
       <c r="B133" s="1" t="n">
@@ -3318,7 +3361,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>运行迁移</t>
+          <t>资源整合</t>
         </is>
       </c>
       <c r="B134" s="1" t="n">
@@ -3328,7 +3371,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>销售转化</t>
+          <t>赞助沟通</t>
         </is>
       </c>
       <c r="B135" s="1" t="n">
@@ -3338,7 +3381,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>问答流程</t>
+          <t>跨文化引导</t>
         </is>
       </c>
       <c r="B136" s="1" t="n">
@@ -3348,7 +3391,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>需求分析</t>
+          <t>转化路径</t>
         </is>
       </c>
       <c r="B137" s="1" t="n">
@@ -3358,7 +3401,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>需求包设计</t>
+          <t>运行迁移</t>
         </is>
       </c>
       <c r="B138" s="1" t="n">
@@ -3368,7 +3411,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>页面规划</t>
+          <t>销售转化</t>
         </is>
       </c>
       <c r="B139" s="1" t="n">
@@ -3378,7 +3421,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>项目包装</t>
+          <t>问答流程</t>
         </is>
       </c>
       <c r="B140" s="1" t="n">
@@ -3388,7 +3431,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>项目对齐</t>
+          <t>需求分析</t>
         </is>
       </c>
       <c r="B141" s="1" t="n">
@@ -3398,7 +3441,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>项目检索</t>
+          <t>需求包设计</t>
         </is>
       </c>
       <c r="B142" s="1" t="n">
@@ -3408,7 +3451,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>风险预案</t>
+          <t>页面规划</t>
         </is>
       </c>
       <c r="B143" s="1" t="n">
@@ -3418,7 +3461,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>验收</t>
+          <t>项目包装</t>
         </is>
       </c>
       <c r="B144" s="1" t="n">
@@ -3428,7 +3471,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>验收清单</t>
+          <t>项目对齐</t>
         </is>
       </c>
       <c r="B145" s="1" t="n">
@@ -3438,15 +3481,205 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
+          <t>项目检索</t>
+        </is>
+      </c>
+      <c r="B146" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="1" t="inlineStr">
+        <is>
+          <t>风险预案</t>
+        </is>
+      </c>
+      <c r="B147" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="1" t="inlineStr">
+        <is>
+          <t>验收</t>
+        </is>
+      </c>
+      <c r="B148" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="1" t="inlineStr">
+        <is>
+          <t>验收清单</t>
+        </is>
+      </c>
+      <c r="B149" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="1" t="inlineStr">
+        <is>
           <t>验收规则</t>
         </is>
       </c>
-      <c r="B146" s="1" t="n">
+      <c r="B150" s="1" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B146"/>
+  <autoFilter ref="A1:B150"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="96" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>类型</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>内容</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>可写结论</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>证据检索 + session 盘点 + 10 产品 AI 优化，保守节省 62.1-144.8 小时。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>可写结论</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>按公开 IT/产品人力成本折算，约 ¥0.75万-¥3.42万。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>潜在收益</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Figma Make 上下文治理约 15.4-26.9 小时/人/12周，需要后续用返工轮次或自动化运行成功率验证。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>测算口径</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>检索提效：952 次路径/产物命中按人工查找时间折算为 23.8-63.5 小时节省。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>测算口径</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>盘点提效：116 条 session 证据按人工阅读、归类、摘录时间折算为 19.3-52.2 小时节省。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>测算口径</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>商品 AI 优化：10 个产品人工优化 20-30 小时与 AI 批量优化 50-60 分钟对比，折算为 19-29.2 小时节省。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>测算口径</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Figma Make 上下文治理：8 份规则文档和 101 条产物证据用于降低补上下文、查错和返工。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>不能硬写</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>当前证据不能证明真实 GMV、真实收入、新增付费客户或新增线索转化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>待补公式</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>新增 GMV = 新增上架商品数 * 单品月 GMV * 提前上线月数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>待补公式</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>新增客户 = 新增线索数 * 转化率，或渠道实际新增客户数。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>